<commit_message>
Agregar retiro autorizado y datos médicos a la ficha de estudiante
Nuevos campos del formulario "Ascend Enrollment" (cols AE-AL y BX-CC),
cargados a mano vía la plantilla de Excel — sin sincronización en vivo
con Google Forms.

- DB (Supabase, tabla students): columna authorized_pickup (jsonb) y
  8 columnas de texto para alergias/condiciones médicas.
- student_template_updated.xlsx: 14 columnas nuevas para la carga
  masiva (8 de salud + 6 de retiro autorizado).
- ExcelUploader.tsx: lee y guarda los campos nuevos al crear/actualizar
  un estudiante; si una fila no trae datos de retiro autorizado, no
  pisa lo que ya estaba guardado.
- students/page.tsx: dos secciones nuevas en el modal de ficha —
  "Alergias y Condiciones Médicas" (solo muestra lo que tiene datos) y
  "Personas Autorizadas para Retirar" (con agregar/quitar directo, sin
  pantalla propia como los padres).
- I18nContext.tsx: labels ES/EN para ambas secciones.
</commit_message>
<xml_diff>
--- a/web/public/student_template_updated.xlsx
+++ b/web/public/student_template_updated.xlsx
@@ -1,52 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Students" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -65,13 +42,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -396,56 +440,157 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AB1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>student_id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>first_name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>last_name</v>
-      </c>
-      <c r="D1" t="str">
-        <v>current_grade</v>
-      </c>
-      <c r="E1" t="str">
-        <v>age</v>
-      </c>
-      <c r="F1" t="str">
-        <v>instrument</v>
-      </c>
-      <c r="G1" t="str">
-        <v>instrument_size</v>
-      </c>
-      <c r="H1" t="str">
-        <v>orchestra_position</v>
-      </c>
-      <c r="I1" t="str">
-        <v>active</v>
-      </c>
-      <c r="J1" t="str">
-        <v>parent_first_name</v>
-      </c>
-      <c r="K1" t="str">
-        <v>parent_last_name</v>
-      </c>
-      <c r="L1" t="str">
-        <v>parent_phone_number</v>
-      </c>
-      <c r="M1" t="str">
-        <v>parent_email</v>
-      </c>
-      <c r="N1" t="str">
-        <v>parent_preferred_contact_method</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>student_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>first_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>last_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>current_grade</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>instrument</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>instrument_size</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>orchestra_position</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>parent_first_name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>parent_last_name</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>parent_phone_number</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>parent_email</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>parent_preferred_contact_method</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>dietary_restrictions</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>dietary_restrictions_details</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>requires_special_care</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>special_care_details</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>takes_medication</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>medication_details</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>has_allergies_or_illness</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>allergies_illness_details</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>authorized_pickup_1_first_name</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>authorized_pickup_1_last_name</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>authorized_pickup_1_phone</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>authorized_pickup_2_first_name</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>authorized_pickup_2_last_name</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>authorized_pickup_2_phone</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>